<commit_message>
created new retrieve function in data-raw
</commit_message>
<xml_diff>
--- a/data-raw/usgs/usgs_corr_table.xlsx
+++ b/data-raw/usgs/usgs_corr_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rsericerca-my.sharepoint.com/personal/mela_rse-web_it/Documents/R/miei_pacchetti/clccr/data-raw/usgs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{949868B5-05C6-4D57-AC27-8919FE4B9135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{949868B5-05C6-4D57-AC27-8919FE4B9135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45656F52-9A36-4BE9-9A4B-DBA9262A0813}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{057858A8-06CC-41A7-9F91-C01C1BC85544}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="23040" windowHeight="12120" xr2:uid="{057858A8-06CC-41A7-9F91-C01C1BC85544}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -305,9 +305,6 @@
     <t>123_USGS</t>
   </si>
   <si>
-    <t>Price, average unit value, ex-works, dollars per metric ton: Fuller’s earth</t>
-  </si>
-  <si>
     <t>Gallium</t>
   </si>
   <si>
@@ -536,9 +533,6 @@
     <t>230_USGS</t>
   </si>
   <si>
-    <t>Nitrogen (Fixed)—Ammonia</t>
-  </si>
-  <si>
     <t>Price, average, free on board Gulf Coast, dollars per short ton</t>
   </si>
   <si>
@@ -900,6 +894,12 @@
   </si>
   <si>
     <t>Price, range of value, dollars per metric ton</t>
+  </si>
+  <si>
+    <t>Price, average unit value, ex-works, dollars per metric ton: Fuller\x92s earth</t>
+  </si>
+  <si>
+    <t>Nitrogen (Fixed)\x97Ammonia</t>
   </si>
 </sst>
 </file>
@@ -935,8 +935,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1273,6 +1274,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9064F1B2-E4D3-4906-95CF-3127663A1305}">
   <dimension ref="A1:E89"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="49.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1709,8 +1713,8 @@
       <c r="C26" t="s">
         <v>55</v>
       </c>
-      <c r="D26" t="s">
-        <v>88</v>
+      <c r="D26" s="1" t="s">
+        <v>285</v>
       </c>
       <c r="E26" t="s">
         <v>15</v>
@@ -1718,16 +1722,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
         <v>89</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" t="s">
         <v>90</v>
-      </c>
-      <c r="C27" t="s">
-        <v>89</v>
-      </c>
-      <c r="D27" t="s">
-        <v>91</v>
       </c>
       <c r="E27" t="s">
         <v>22</v>
@@ -1735,16 +1739,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" t="s">
         <v>92</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>93</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>94</v>
-      </c>
-      <c r="D28" t="s">
-        <v>95</v>
       </c>
       <c r="E28" t="s">
         <v>15</v>
@@ -1752,16 +1756,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" t="s">
         <v>96</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" t="s">
         <v>97</v>
-      </c>
-      <c r="C29" t="s">
-        <v>96</v>
-      </c>
-      <c r="D29" t="s">
-        <v>98</v>
       </c>
       <c r="E29" t="s">
         <v>22</v>
@@ -1769,16 +1773,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" t="s">
         <v>99</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>100</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>101</v>
-      </c>
-      <c r="D30" t="s">
-        <v>102</v>
       </c>
       <c r="E30" t="s">
         <v>15</v>
@@ -1786,13 +1790,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" t="s">
         <v>103</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>104</v>
-      </c>
-      <c r="C31" t="s">
-        <v>105</v>
       </c>
       <c r="D31" t="s">
         <v>38</v>
@@ -1803,16 +1807,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" t="s">
         <v>106</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
+        <v>105</v>
+      </c>
+      <c r="D32" t="s">
         <v>107</v>
-      </c>
-      <c r="C32" t="s">
-        <v>106</v>
-      </c>
-      <c r="D32" t="s">
-        <v>108</v>
       </c>
       <c r="E32" t="s">
         <v>15</v>
@@ -1820,16 +1824,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" t="s">
         <v>109</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
+        <v>108</v>
+      </c>
+      <c r="D33" t="s">
         <v>110</v>
-      </c>
-      <c r="C33" t="s">
-        <v>109</v>
-      </c>
-      <c r="D33" t="s">
-        <v>111</v>
       </c>
       <c r="E33" t="s">
         <v>22</v>
@@ -1837,16 +1841,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" t="s">
         <v>112</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>113</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>114</v>
-      </c>
-      <c r="D34" t="s">
-        <v>115</v>
       </c>
       <c r="E34" t="s">
         <v>15</v>
@@ -1854,16 +1858,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>115</v>
+      </c>
+      <c r="B35" t="s">
         <v>116</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" t="s">
         <v>117</v>
-      </c>
-      <c r="C35" t="s">
-        <v>116</v>
-      </c>
-      <c r="D35" t="s">
-        <v>118</v>
       </c>
       <c r="E35" t="s">
         <v>22</v>
@@ -1871,16 +1875,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" t="s">
         <v>119</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" t="s">
         <v>120</v>
-      </c>
-      <c r="C36" t="s">
-        <v>119</v>
-      </c>
-      <c r="D36" t="s">
-        <v>121</v>
       </c>
       <c r="E36" t="s">
         <v>22</v>
@@ -1888,33 +1892,33 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>121</v>
+      </c>
+      <c r="B37" t="s">
         <v>122</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>121</v>
+      </c>
+      <c r="D37" t="s">
         <v>123</v>
       </c>
-      <c r="C37" t="s">
-        <v>122</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>124</v>
-      </c>
-      <c r="E37" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>125</v>
+      </c>
+      <c r="B38" t="s">
         <v>126</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>127</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>128</v>
-      </c>
-      <c r="D38" t="s">
-        <v>129</v>
       </c>
       <c r="E38" t="s">
         <v>15</v>
@@ -1922,16 +1926,16 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>129</v>
+      </c>
+      <c r="B39" t="s">
         <v>130</v>
-      </c>
-      <c r="B39" t="s">
-        <v>131</v>
       </c>
       <c r="C39" t="s">
         <v>55</v>
       </c>
       <c r="D39" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E39" t="s">
         <v>15</v>
@@ -1939,16 +1943,16 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>132</v>
+      </c>
+      <c r="B40" t="s">
         <v>133</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>134</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>135</v>
-      </c>
-      <c r="D40" t="s">
-        <v>136</v>
       </c>
       <c r="E40" t="s">
         <v>15</v>
@@ -1956,16 +1960,16 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" t="s">
         <v>137</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
+        <v>136</v>
+      </c>
+      <c r="D41" t="s">
         <v>138</v>
-      </c>
-      <c r="C41" t="s">
-        <v>137</v>
-      </c>
-      <c r="D41" t="s">
-        <v>139</v>
       </c>
       <c r="E41" t="s">
         <v>22</v>
@@ -1973,10 +1977,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42" t="s">
         <v>140</v>
-      </c>
-      <c r="B42" t="s">
-        <v>141</v>
       </c>
       <c r="C42" t="s">
         <v>37</v>
@@ -1990,16 +1994,16 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" t="s">
         <v>142</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>143</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>144</v>
-      </c>
-      <c r="D43" t="s">
-        <v>145</v>
       </c>
       <c r="E43" t="s">
         <v>15</v>
@@ -2007,16 +2011,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>145</v>
+      </c>
+      <c r="B44" t="s">
         <v>146</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>147</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>148</v>
-      </c>
-      <c r="D44" t="s">
-        <v>149</v>
       </c>
       <c r="E44" t="s">
         <v>15</v>
@@ -2024,16 +2028,16 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>149</v>
+      </c>
+      <c r="B45" t="s">
         <v>150</v>
       </c>
-      <c r="B45" t="s">
-        <v>151</v>
-      </c>
       <c r="C45" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E45" t="s">
         <v>22</v>
@@ -2041,16 +2045,16 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>151</v>
+      </c>
+      <c r="B46" t="s">
         <v>152</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" t="s">
         <v>153</v>
-      </c>
-      <c r="C46" t="s">
-        <v>152</v>
-      </c>
-      <c r="D46" t="s">
-        <v>154</v>
       </c>
       <c r="E46" t="s">
         <v>22</v>
@@ -2058,16 +2062,16 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>154</v>
+      </c>
+      <c r="B47" t="s">
         <v>155</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>156</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>157</v>
-      </c>
-      <c r="D47" t="s">
-        <v>158</v>
       </c>
       <c r="E47" t="s">
         <v>15</v>
@@ -2075,16 +2079,16 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>158</v>
+      </c>
+      <c r="B48" t="s">
         <v>159</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>160</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>161</v>
-      </c>
-      <c r="D48" t="s">
-        <v>162</v>
       </c>
       <c r="E48" t="s">
         <v>22</v>
@@ -2092,33 +2096,33 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>162</v>
+      </c>
+      <c r="B49" t="s">
         <v>163</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
+        <v>286</v>
+      </c>
+      <c r="D49" t="s">
         <v>164</v>
       </c>
-      <c r="C49" t="s">
+      <c r="E49" t="s">
         <v>165</v>
-      </c>
-      <c r="D49" t="s">
-        <v>166</v>
-      </c>
-      <c r="E49" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>166</v>
+      </c>
+      <c r="B50" t="s">
+        <v>167</v>
+      </c>
+      <c r="C50" t="s">
+        <v>166</v>
+      </c>
+      <c r="D50" t="s">
         <v>168</v>
-      </c>
-      <c r="B50" t="s">
-        <v>169</v>
-      </c>
-      <c r="C50" t="s">
-        <v>168</v>
-      </c>
-      <c r="D50" t="s">
-        <v>170</v>
       </c>
       <c r="E50" t="s">
         <v>15</v>
@@ -2126,16 +2130,16 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>169</v>
+      </c>
+      <c r="B51" t="s">
+        <v>170</v>
+      </c>
+      <c r="C51" t="s">
+        <v>169</v>
+      </c>
+      <c r="D51" t="s">
         <v>171</v>
-      </c>
-      <c r="B51" t="s">
-        <v>172</v>
-      </c>
-      <c r="C51" t="s">
-        <v>171</v>
-      </c>
-      <c r="D51" t="s">
-        <v>173</v>
       </c>
       <c r="E51" t="s">
         <v>15</v>
@@ -2143,16 +2147,16 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>172</v>
+      </c>
+      <c r="B52" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" t="s">
         <v>174</v>
       </c>
-      <c r="B52" t="s">
+      <c r="D52" t="s">
         <v>175</v>
-      </c>
-      <c r="C52" t="s">
-        <v>176</v>
-      </c>
-      <c r="D52" t="s">
-        <v>177</v>
       </c>
       <c r="E52" t="s">
         <v>15</v>
@@ -2160,16 +2164,16 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>176</v>
+      </c>
+      <c r="B53" t="s">
+        <v>177</v>
+      </c>
+      <c r="C53" t="s">
         <v>178</v>
       </c>
-      <c r="B53" t="s">
+      <c r="D53" t="s">
         <v>179</v>
-      </c>
-      <c r="C53" t="s">
-        <v>180</v>
-      </c>
-      <c r="D53" t="s">
-        <v>181</v>
       </c>
       <c r="E53" t="s">
         <v>15</v>
@@ -2177,16 +2181,16 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>180</v>
+      </c>
+      <c r="B54" t="s">
+        <v>181</v>
+      </c>
+      <c r="C54" t="s">
         <v>182</v>
       </c>
-      <c r="B54" t="s">
+      <c r="D54" t="s">
         <v>183</v>
-      </c>
-      <c r="C54" t="s">
-        <v>184</v>
-      </c>
-      <c r="D54" t="s">
-        <v>185</v>
       </c>
       <c r="E54" t="s">
         <v>15</v>
@@ -2194,16 +2198,16 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>184</v>
+      </c>
+      <c r="B55" t="s">
+        <v>185</v>
+      </c>
+      <c r="C55" t="s">
+        <v>184</v>
+      </c>
+      <c r="D55" t="s">
         <v>186</v>
-      </c>
-      <c r="B55" t="s">
-        <v>187</v>
-      </c>
-      <c r="C55" t="s">
-        <v>186</v>
-      </c>
-      <c r="D55" t="s">
-        <v>188</v>
       </c>
       <c r="E55" t="s">
         <v>22</v>
@@ -2211,118 +2215,118 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>187</v>
+      </c>
+      <c r="B56" t="s">
+        <v>188</v>
+      </c>
+      <c r="C56" t="s">
+        <v>187</v>
+      </c>
+      <c r="D56" t="s">
         <v>189</v>
       </c>
-      <c r="B56" t="s">
-        <v>190</v>
-      </c>
-      <c r="C56" t="s">
-        <v>189</v>
-      </c>
-      <c r="D56" t="s">
-        <v>191</v>
-      </c>
       <c r="E56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B57" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C57" t="s">
+        <v>187</v>
+      </c>
+      <c r="D57" t="s">
         <v>189</v>
       </c>
-      <c r="D57" t="s">
-        <v>191</v>
-      </c>
       <c r="E57" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B58" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C58" t="s">
+        <v>187</v>
+      </c>
+      <c r="D58" t="s">
         <v>189</v>
       </c>
-      <c r="D58" t="s">
-        <v>191</v>
-      </c>
       <c r="E58" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B59" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C59" t="s">
+        <v>187</v>
+      </c>
+      <c r="D59" t="s">
         <v>189</v>
       </c>
-      <c r="D59" t="s">
-        <v>191</v>
-      </c>
       <c r="E59" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B60" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C60" t="s">
+        <v>187</v>
+      </c>
+      <c r="D60" t="s">
         <v>189</v>
       </c>
-      <c r="D60" t="s">
-        <v>191</v>
-      </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>198</v>
+      </c>
+      <c r="B61" t="s">
+        <v>199</v>
+      </c>
+      <c r="C61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D61" t="s">
         <v>200</v>
       </c>
-      <c r="B61" t="s">
-        <v>201</v>
-      </c>
-      <c r="C61" t="s">
-        <v>200</v>
-      </c>
-      <c r="D61" t="s">
-        <v>202</v>
-      </c>
       <c r="E61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" t="s">
+        <v>202</v>
+      </c>
+      <c r="C62" t="s">
+        <v>113</v>
+      </c>
+      <c r="D62" t="s">
         <v>203</v>
-      </c>
-      <c r="B62" t="s">
-        <v>204</v>
-      </c>
-      <c r="C62" t="s">
-        <v>114</v>
-      </c>
-      <c r="D62" t="s">
-        <v>205</v>
       </c>
       <c r="E62" t="s">
         <v>15</v>
@@ -2330,13 +2334,13 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B63" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C63" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D63" t="s">
         <v>38</v>
@@ -2347,10 +2351,10 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C64" t="s">
         <v>37</v>
@@ -2364,16 +2368,16 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
+        <v>208</v>
+      </c>
+      <c r="B65" t="s">
+        <v>209</v>
+      </c>
+      <c r="C65" t="s">
+        <v>208</v>
+      </c>
+      <c r="D65" t="s">
         <v>210</v>
-      </c>
-      <c r="B65" t="s">
-        <v>211</v>
-      </c>
-      <c r="C65" t="s">
-        <v>210</v>
-      </c>
-      <c r="D65" t="s">
-        <v>212</v>
       </c>
       <c r="E65" t="s">
         <v>22</v>
@@ -2381,16 +2385,16 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>211</v>
+      </c>
+      <c r="B66" t="s">
+        <v>212</v>
+      </c>
+      <c r="C66" t="s">
+        <v>211</v>
+      </c>
+      <c r="D66" t="s">
         <v>213</v>
-      </c>
-      <c r="B66" t="s">
-        <v>214</v>
-      </c>
-      <c r="C66" t="s">
-        <v>213</v>
-      </c>
-      <c r="D66" t="s">
-        <v>215</v>
       </c>
       <c r="E66" t="s">
         <v>22</v>
@@ -2398,16 +2402,16 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>214</v>
+      </c>
+      <c r="B67" t="s">
+        <v>215</v>
+      </c>
+      <c r="C67" t="s">
         <v>216</v>
       </c>
-      <c r="B67" t="s">
+      <c r="D67" t="s">
         <v>217</v>
-      </c>
-      <c r="C67" t="s">
-        <v>218</v>
-      </c>
-      <c r="D67" t="s">
-        <v>219</v>
       </c>
       <c r="E67" t="s">
         <v>15</v>
@@ -2415,16 +2419,16 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>218</v>
+      </c>
+      <c r="B68" t="s">
+        <v>219</v>
+      </c>
+      <c r="C68" t="s">
         <v>220</v>
       </c>
-      <c r="B68" t="s">
+      <c r="D68" t="s">
         <v>221</v>
-      </c>
-      <c r="C68" t="s">
-        <v>222</v>
-      </c>
-      <c r="D68" t="s">
-        <v>223</v>
       </c>
       <c r="E68" t="s">
         <v>15</v>
@@ -2432,16 +2436,16 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
+        <v>222</v>
+      </c>
+      <c r="B69" t="s">
+        <v>223</v>
+      </c>
+      <c r="C69" t="s">
+        <v>222</v>
+      </c>
+      <c r="D69" t="s">
         <v>224</v>
-      </c>
-      <c r="B69" t="s">
-        <v>225</v>
-      </c>
-      <c r="C69" t="s">
-        <v>224</v>
-      </c>
-      <c r="D69" t="s">
-        <v>226</v>
       </c>
       <c r="E69" t="s">
         <v>52</v>
@@ -2449,16 +2453,16 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
+        <v>225</v>
+      </c>
+      <c r="B70" t="s">
+        <v>226</v>
+      </c>
+      <c r="C70" t="s">
+        <v>225</v>
+      </c>
+      <c r="D70" t="s">
         <v>227</v>
-      </c>
-      <c r="B70" t="s">
-        <v>228</v>
-      </c>
-      <c r="C70" t="s">
-        <v>227</v>
-      </c>
-      <c r="D70" t="s">
-        <v>229</v>
       </c>
       <c r="E70" t="s">
         <v>15</v>
@@ -2466,16 +2470,16 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
+        <v>228</v>
+      </c>
+      <c r="B71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C71" t="s">
         <v>230</v>
       </c>
-      <c r="B71" t="s">
+      <c r="D71" t="s">
         <v>231</v>
-      </c>
-      <c r="C71" t="s">
-        <v>232</v>
-      </c>
-      <c r="D71" t="s">
-        <v>233</v>
       </c>
       <c r="E71" t="s">
         <v>15</v>
@@ -2483,16 +2487,16 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
+        <v>232</v>
+      </c>
+      <c r="B72" t="s">
+        <v>233</v>
+      </c>
+      <c r="C72" t="s">
+        <v>232</v>
+      </c>
+      <c r="D72" t="s">
         <v>234</v>
-      </c>
-      <c r="B72" t="s">
-        <v>235</v>
-      </c>
-      <c r="C72" t="s">
-        <v>234</v>
-      </c>
-      <c r="D72" t="s">
-        <v>236</v>
       </c>
       <c r="E72" t="s">
         <v>22</v>
@@ -2500,16 +2504,16 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B73" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C73" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D73" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E73" t="s">
         <v>22</v>
@@ -2517,16 +2521,16 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>237</v>
+      </c>
+      <c r="B74" t="s">
+        <v>238</v>
+      </c>
+      <c r="C74" t="s">
+        <v>237</v>
+      </c>
+      <c r="D74" t="s">
         <v>239</v>
-      </c>
-      <c r="B74" t="s">
-        <v>240</v>
-      </c>
-      <c r="C74" t="s">
-        <v>239</v>
-      </c>
-      <c r="D74" t="s">
-        <v>241</v>
       </c>
       <c r="E74" t="s">
         <v>22</v>
@@ -2534,16 +2538,16 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
+        <v>240</v>
+      </c>
+      <c r="B75" t="s">
+        <v>241</v>
+      </c>
+      <c r="C75" t="s">
+        <v>240</v>
+      </c>
+      <c r="D75" t="s">
         <v>242</v>
-      </c>
-      <c r="B75" t="s">
-        <v>243</v>
-      </c>
-      <c r="C75" t="s">
-        <v>242</v>
-      </c>
-      <c r="D75" t="s">
-        <v>244</v>
       </c>
       <c r="E75" t="s">
         <v>22</v>
@@ -2551,16 +2555,16 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>243</v>
+      </c>
+      <c r="B76" t="s">
+        <v>244</v>
+      </c>
+      <c r="C76" t="s">
+        <v>243</v>
+      </c>
+      <c r="D76" t="s">
         <v>245</v>
-      </c>
-      <c r="B76" t="s">
-        <v>246</v>
-      </c>
-      <c r="C76" t="s">
-        <v>245</v>
-      </c>
-      <c r="D76" t="s">
-        <v>247</v>
       </c>
       <c r="E76" t="s">
         <v>22</v>
@@ -2568,16 +2572,16 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
+        <v>246</v>
+      </c>
+      <c r="B77" t="s">
+        <v>247</v>
+      </c>
+      <c r="C77" t="s">
         <v>248</v>
       </c>
-      <c r="B77" t="s">
+      <c r="D77" t="s">
         <v>249</v>
-      </c>
-      <c r="C77" t="s">
-        <v>250</v>
-      </c>
-      <c r="D77" t="s">
-        <v>251</v>
       </c>
       <c r="E77" t="s">
         <v>15</v>
@@ -2585,16 +2589,16 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B78" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C78" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D78" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E78" t="s">
         <v>15</v>
@@ -2602,16 +2606,16 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B79" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C79" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D79" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E79" t="s">
         <v>15</v>
@@ -2619,16 +2623,16 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B80" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C80" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D80" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E80" t="s">
         <v>15</v>
@@ -2636,16 +2640,16 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
+        <v>256</v>
+      </c>
+      <c r="B81" t="s">
+        <v>257</v>
+      </c>
+      <c r="C81" t="s">
         <v>258</v>
       </c>
-      <c r="B81" t="s">
+      <c r="D81" t="s">
         <v>259</v>
-      </c>
-      <c r="C81" t="s">
-        <v>260</v>
-      </c>
-      <c r="D81" t="s">
-        <v>261</v>
       </c>
       <c r="E81" t="s">
         <v>22</v>
@@ -2653,16 +2657,16 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B82" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C82" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D82" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E82" t="s">
         <v>15</v>
@@ -2670,16 +2674,16 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
+        <v>262</v>
+      </c>
+      <c r="B83" t="s">
+        <v>263</v>
+      </c>
+      <c r="C83" t="s">
+        <v>113</v>
+      </c>
+      <c r="D83" t="s">
         <v>264</v>
-      </c>
-      <c r="B83" t="s">
-        <v>265</v>
-      </c>
-      <c r="C83" t="s">
-        <v>114</v>
-      </c>
-      <c r="D83" t="s">
-        <v>266</v>
       </c>
       <c r="E83" t="s">
         <v>15</v>
@@ -2687,33 +2691,33 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
+        <v>265</v>
+      </c>
+      <c r="B84" t="s">
+        <v>266</v>
+      </c>
+      <c r="C84" t="s">
+        <v>265</v>
+      </c>
+      <c r="D84" t="s">
         <v>267</v>
       </c>
-      <c r="B84" t="s">
+      <c r="E84" t="s">
         <v>268</v>
-      </c>
-      <c r="C84" t="s">
-        <v>267</v>
-      </c>
-      <c r="D84" t="s">
-        <v>269</v>
-      </c>
-      <c r="E84" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
+        <v>269</v>
+      </c>
+      <c r="B85" t="s">
+        <v>270</v>
+      </c>
+      <c r="C85" t="s">
+        <v>269</v>
+      </c>
+      <c r="D85" t="s">
         <v>271</v>
-      </c>
-      <c r="B85" t="s">
-        <v>272</v>
-      </c>
-      <c r="C85" t="s">
-        <v>271</v>
-      </c>
-      <c r="D85" t="s">
-        <v>273</v>
       </c>
       <c r="E85" t="s">
         <v>22</v>
@@ -2721,16 +2725,16 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
+        <v>272</v>
+      </c>
+      <c r="B86" t="s">
+        <v>273</v>
+      </c>
+      <c r="C86" t="s">
+        <v>272</v>
+      </c>
+      <c r="D86" t="s">
         <v>274</v>
-      </c>
-      <c r="B86" t="s">
-        <v>275</v>
-      </c>
-      <c r="C86" t="s">
-        <v>274</v>
-      </c>
-      <c r="D86" t="s">
-        <v>276</v>
       </c>
       <c r="E86" t="s">
         <v>22</v>
@@ -2738,41 +2742,41 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
+        <v>275</v>
+      </c>
+      <c r="B87" t="s">
+        <v>276</v>
+      </c>
+      <c r="C87" t="s">
+        <v>275</v>
+      </c>
+      <c r="D87" t="s">
         <v>277</v>
       </c>
-      <c r="B87" t="s">
+      <c r="E87" t="s">
         <v>278</v>
-      </c>
-      <c r="C87" t="s">
-        <v>277</v>
-      </c>
-      <c r="D87" t="s">
-        <v>279</v>
-      </c>
-      <c r="E87" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B88" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
+        <v>281</v>
+      </c>
+      <c r="B89" t="s">
+        <v>282</v>
+      </c>
+      <c r="C89" t="s">
         <v>283</v>
       </c>
-      <c r="B89" t="s">
+      <c r="D89" t="s">
         <v>284</v>
-      </c>
-      <c r="C89" t="s">
-        <v>285</v>
-      </c>
-      <c r="D89" t="s">
-        <v>286</v>
       </c>
       <c r="E89" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
fixed bug in data preparation: scandium price was not properly loaded
</commit_message>
<xml_diff>
--- a/data-raw/usgs/usgs_corr_table.xlsx
+++ b/data-raw/usgs/usgs_corr_table.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="13" documentId="8_{949868B5-05C6-4D57-AC27-8919FE4B9135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45656F52-9A36-4BE9-9A4B-DBA9262A0813}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="23040" windowHeight="12120" xr2:uid="{057858A8-06CC-41A7-9F91-C01C1BC85544}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{057858A8-06CC-41A7-9F91-C01C1BC85544}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -935,9 +935,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1713,7 +1712,7 @@
       <c r="C26" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>285</v>
       </c>
       <c r="E26" t="s">

</xml_diff>